<commit_message>
Last Sync: 2026-01-05 09:32 (Mobile)
</commit_message>
<xml_diff>
--- a/Courses/Term 3/QAM-III/601 DATA Caps - Price Qty Cost profit.xlsx
+++ b/Courses/Term 3/QAM-III/601 DATA Caps - Price Qty Cost profit.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/suranjandas/Desktop/SIRMAUR. IIM .. Nov 14 2025/T1 - Non Linear Programming/Data to students - Email/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31B53793-64AD-A743-AB43-3CB52D4C966A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1076737D-8F77-594A-B147-D3BA723A1948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1760" yWindow="1320" windowWidth="27640" windowHeight="16760" xr2:uid="{B2BED8D6-8C7E-0E42-9D17-93C443EBC8CA}"/>
   </bookViews>
   <sheets>
     <sheet name="601 caps Exp()" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,6 +27,7 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>The Selling Price for a monkey cap varies within the range of $5 to $20 based on Demand conditions driven by the weather and customer preference.</t>
   </si>
@@ -68,13 +69,28 @@
   <si>
     <t>What is the Price at which you will a) Maximize revenue b) Mamimize profit?</t>
   </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t>PROFIT</t>
+  </si>
+  <si>
+    <t>COGS</t>
+  </si>
+  <si>
+    <t>DEMAND</t>
+  </si>
+  <si>
+    <t>QTY</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="8" formatCode="&quot;₹&quot;#,##0.00_);[Red]\(&quot;₹&quot;#,##0.00\)"/>
+    <numFmt numFmtId="164" formatCode="&quot;₹&quot;#,##0.00_);[Red]\(&quot;₹&quot;#,##0.00\)"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -127,7 +143,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -149,9 +165,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -189,7 +205,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -295,7 +311,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -437,7 +453,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -445,8 +461,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{309BED9E-3E41-FF4D-B485-F8C73E39BF82}">
-  <dimension ref="A1:Q11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:Q24"/>
+  <sheetFormatPr defaultColWidth="10.8515625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="11.58984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.58984375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -488,7 +508,7 @@
       <c r="L6" s="2"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="8" spans="1:17" ht="20" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" ht="21" x14ac:dyDescent="0.2">
       <c r="C8" s="4" t="s">
         <v>4</v>
       </c>
@@ -496,6 +516,92 @@
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B13">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14">
+        <v>5</v>
+      </c>
+      <c r="F14" t="s">
+        <v>8</v>
+      </c>
+      <c r="G14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15">
+        <f>B13-B14</f>
+        <v>2</v>
+      </c>
+      <c r="G15">
+        <v>496.58530380000002</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="F16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17">
+        <f>1000*EXP(-0.1*B13)</f>
+        <v>496.58530379140944</v>
+      </c>
+      <c r="F17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F18">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F19">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F20">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F21">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F22">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F23">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F24">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>